<commit_message>
Esimerkki-Excel anonymisoitu, päivitys ei korvaa käyttäjän Exceliä
- Opintosuunnitelmat.xlsx: YTO- ja Väylä-välilehtien opettajien nimet (11 tekstiä, 18 solua)
  korvattu merkinnällä "(vastuuopettaja)". Vain xl/sharedStrings.xml muuttui; muotoilut ja
  välilehdet ovat ennallaan.
- Varmistettu testillä, että päivitys ei korvaa käyttäjän asetuskansiossa olevaa Exceliä eikä
  config.jsonia: uusi pohja kopioidaan vain, jos käyttäjällä ei vielä ole tiedostoa.
  Periaate kirjattu ensure_user_filesiin ja README:n Päivitys-osioon.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Opintosuunnitelmat.xlsx
+++ b/Opintosuunnitelmat.xlsx
@@ -88,7 +88,7 @@
     <t>Järjestelmätuessa toimiminen</t>
   </si>
   <si>
-    <t>Ilmoittaudu väylälle. Pyydä tehtävät opettajalta (Damien Kuosmanen)</t>
+    <t>Ilmoittaudu väylälle. Pyydä tehtävät opettajalta (vastuuopettaja)</t>
   </si>
   <si>
     <t>Tietoteknisen ratkaisun myynti</t>
@@ -103,7 +103,7 @@
     <t>Äidinkieli / S2</t>
   </si>
   <si>
-    <t>Avoin (Päivi Honkala)</t>
+    <t>Avoin (vastuuopettaja)</t>
   </si>
   <si>
     <t>Ruotsi</t>
@@ -157,37 +157,37 @@
     <t>Unix-komentorivin perusteet (valinnainen)</t>
   </si>
   <si>
-    <t>Joustava (Edward Krogius)</t>
+    <t>Joustava (vastuuopettaja)</t>
   </si>
   <si>
     <t>Tulee osana tieto- ja viestintätekniikan perustehtäviä</t>
   </si>
   <si>
-    <t>Joustava (Elina Kuutti)</t>
-  </si>
-  <si>
-    <t>Avoin (Mika Kurki)</t>
-  </si>
-  <si>
-    <t>Joustava (Matti Seise / Antti Honkasalo)</t>
-  </si>
-  <si>
-    <t>Avoin (Petteri Kärkkäinen)</t>
+    <t>Joustava (vastuuopettaja)</t>
+  </si>
+  <si>
+    <t>Avoin (vastuuopettaja)</t>
+  </si>
+  <si>
+    <t>Joustava (vastuuopettaja)</t>
+  </si>
+  <si>
+    <t>Avoin (vastuuopettaja)</t>
   </si>
   <si>
     <t>Lukio-opintojen suorittaminen TYK:issä</t>
   </si>
   <si>
-    <t>Avoin 2018 PAK Yhteiskunnassa ja kansalaisena toimiminen (Piritta Pyykönen)</t>
-  </si>
-  <si>
-    <t>Avoin 2020 PAK Yrittäjyys ja yrittäjämäinen toiminta (Piritta Pyykönen)</t>
-  </si>
-  <si>
-    <t>Avoin 2018 PAK Työkyvyn ja hyvinvoinnin ylläpit., terveystieto &amp; Avoin 2018 PAK Työkyvyn ja hyvinvoinnin ylläpitäminen, liikunta (Petteri Kärkkäinen)</t>
-  </si>
-  <si>
-    <t>Avoin 2018 PAK Kestävän kehityksen edistäminen, pakollinen (Tuomas Kalliokoski)</t>
+    <t>Avoin 2018 PAK Yhteiskunnassa ja kansalaisena toimiminen (vastuuopettaja)</t>
+  </si>
+  <si>
+    <t>Avoin 2020 PAK Yrittäjyys ja yrittäjämäinen toiminta (vastuuopettaja)</t>
+  </si>
+  <si>
+    <t>Avoin 2018 PAK Työkyvyn ja hyvinvoinnin ylläpit., terveystieto &amp; Avoin 2018 PAK Työkyvyn ja hyvinvoinnin ylläpitäminen, liikunta (vastuuopettaja)</t>
+  </si>
+  <si>
+    <t>Avoin 2018 PAK Kestävän kehityksen edistäminen, pakollinen (vastuuopettaja)</t>
   </si>
 </sst>
 </file>

</xml_diff>